<commit_message>
feat(qa): tampilkan seed --sample di output + dokumentasi reproduksi run identik
SAMPLE_SEED (20260816) jadi konstanta bernama; random_statuses memakainya
sebagai default dan nilai seed dicetak di output --sample. QA Test Plan §8.1
mendokumentasikan cara mereproduksi run --sample yang sama persis (seed tetap,
pin QA_RUN_DATE/QA_ENVIRONMENT untuk byte-identik lintas hari, verifikasi
sha256 CSV/JSON; XLSX dibandingkan via isi sel karena timestamp zip openpyxl).
Artefak sample di-regenerasi (run date 2026-08-18).

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/qa-test-cases-sample.xlsx
+++ b/qa-test-cases-sample.xlsx
@@ -682,7 +682,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -4738,7 +4738,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -5284,7 +5284,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
@@ -5674,7 +5674,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
@@ -6610,7 +6610,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
@@ -6688,7 +6688,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
@@ -6844,7 +6844,7 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
@@ -6922,7 +6922,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
@@ -7000,7 +7000,7 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -7390,7 +7390,7 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
@@ -7702,7 +7702,7 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -8162,7 +8162,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr">
@@ -8318,7 +8318,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr">
@@ -8396,7 +8396,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K102" s="2" t="inlineStr">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
@@ -8630,7 +8630,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr">
@@ -8786,7 +8786,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
@@ -8942,7 +8942,7 @@
       </c>
       <c r="J108" s="6" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K108" s="6" t="inlineStr">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="J111" s="6" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K111" s="6" t="inlineStr">
@@ -9254,7 +9254,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K113" s="2" t="inlineStr">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K115" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K116" s="2" t="inlineStr">
@@ -9644,7 +9644,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr">
@@ -9722,7 +9722,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr">
@@ -9800,7 +9800,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K120" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K121" s="2" t="inlineStr">
@@ -10034,7 +10034,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K122" s="2" t="inlineStr">
@@ -10112,7 +10112,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K124" s="2" t="inlineStr">
@@ -10268,7 +10268,7 @@
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K125" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K126" s="2" t="inlineStr">
@@ -10424,7 +10424,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K128" s="2" t="inlineStr">
@@ -10580,7 +10580,7 @@
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K129" s="2" t="inlineStr">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K130" s="2" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K131" s="2" t="inlineStr">
@@ -10814,7 +10814,7 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K132" s="2" t="inlineStr">
@@ -10892,7 +10892,7 @@
       </c>
       <c r="J133" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K133" s="2" t="inlineStr">
@@ -10970,7 +10970,7 @@
       </c>
       <c r="J134" s="6" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K134" s="6" t="inlineStr">
@@ -11048,7 +11048,7 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K135" s="2" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K136" s="2" t="inlineStr">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K138" s="2" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K139" s="2" t="inlineStr">
@@ -11378,7 +11378,7 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K140" s="2" t="inlineStr">
@@ -11444,7 +11444,7 @@
       </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K141" s="2" t="inlineStr">
@@ -11510,7 +11510,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
@@ -11642,7 +11642,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -11774,7 +11774,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr">
@@ -11840,7 +11840,7 @@
       </c>
       <c r="J147" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K147" s="2" t="inlineStr">
@@ -11918,7 +11918,7 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K148" s="2" t="inlineStr">
@@ -11996,7 +11996,7 @@
       </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K149" s="2" t="inlineStr">
@@ -12074,7 +12074,7 @@
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="K150" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(qa): XLSX byte-deterministik + regenerasi artefak --sample
Pin wb.properties.created/modified ke epoch 2026-01-01T00:00:00Z di
write_xlsx() dan write_results_template_xlsx() agar hash XLSX stabil
antar run (hash stabil = gate qa-sync di CI tidak gagal karena
perbedaan timestamp).

Regenerasi 4 artefak --sample dengan generator terbaru:
- qa-test-cases-sample.xlsx (deterministik)
- qa-test-cases-sample-tracker.csv
- qa-test-results-sample-testrail.csv
- qa-test-results-sample.json

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/qa-test-cases-sample.xlsx
+++ b/qa-test-cases-sample.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$P$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$P$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P150"/>
+  <dimension ref="A1:P153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11873,44 +11873,32 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>TC-CFL-01</t>
+          <t>RG-20</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Arus Kas</t>
+          <t>Skenario Regresi</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>3 seksi arus kas</t>
+          <t>SESSION_EXPIRED — refresh token kedaluwarsa di server</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>1 - Critical</t>
-        </is>
-      </c>
-      <c r="F148" s="3" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="G148" s="2" t="inlineStr">
-        <is>
-          <t>AAJ-028</t>
-        </is>
-      </c>
-      <c r="H148" s="2" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
+          <t>3 - Medium</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr"/>
+      <c r="G148" s="2" t="inlineStr"/>
+      <c r="H148" s="2" t="inlineStr"/>
       <c r="I148" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -11934,61 +11922,49 @@
       <c r="M148" s="2" t="inlineStr"/>
       <c r="N148" s="4" t="inlineStr">
         <is>
-          <t>Buka laporan Arus Kas Maret</t>
+          <t>Login → POST /admin/expire-refresh-tokens (semua refresh token basi) + akses token dipaksa basi → pemicu fetch/reload → auto-refresh gagal 401 SESSION_EXPIRED → modal "Sesi Berakhir" → "Masuk kembali" → login ulang</t>
         </is>
       </c>
       <c r="O148" s="4" t="inlineStr">
         <is>
-          <t>Seksi Operasi / Investasi / Pendanaan dengan subtotal; metode tidak langsung</t>
+          <t>Modal "Sesi Berakhir" muncul (bukan sekadar error inline); logout otomatis — token dibersihkan dari localStorage; login ulang wajib → sesi baru dengan token baru</t>
         </is>
       </c>
       <c r="P148" s="4" t="inlineStr">
         <is>
-          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+          <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>TC-CFL-02</t>
+          <t>RG-21</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Arus Kas</t>
+          <t>Skenario Regresi</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Konsistensi kas</t>
+          <t>RATE_LIMITED — retry otomatis pulih</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>1 - Critical</t>
-        </is>
-      </c>
-      <c r="F149" s="3" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="G149" s="2" t="inlineStr">
-        <is>
-          <t>AAJ-028</t>
-        </is>
-      </c>
-      <c r="H149" s="2" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
+          <t>3 - Medium</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr"/>
+      <c r="G149" s="2" t="inlineStr"/>
+      <c r="H149" s="2" t="inlineStr"/>
       <c r="I149" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -12012,61 +11988,49 @@
       <c r="M149" s="2" t="inlineStr"/>
       <c r="N149" s="4" t="inlineStr">
         <is>
-          <t>Cek formula</t>
+          <t>POST /admin/set-rate-limit (ambang 1 req/endpoint) → simpan jurnal #1 (200) → simpan jurnal #2 kena 429 → klien retry otomatis (jeda Retry-After, cap 5 dtk) → ambang dinaikkan → retry berhasil</t>
         </is>
       </c>
       <c r="O149" s="4" t="inlineStr">
         <is>
-          <t>Kas akhir = kas awal + arus kas bersih (unit test)</t>
+          <t>Jurnal #1 &amp; #2 tersimpan (8 seed + 2); TIDAK ada toast "Terlalu banyak permintaan"; bukti jaringan 429 → retry 201; sesi tetap aktif</t>
         </is>
       </c>
       <c r="P149" s="4" t="inlineStr">
         <is>
-          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+          <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>TC-CFL-03</t>
+          <t>RG-22</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Arus Kas</t>
+          <t>Skenario Regresi</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Mapping grup akun</t>
+          <t>RATE_LIMITED — tetap diblokir</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>2 - High</t>
-        </is>
-      </c>
-      <c r="F150" s="5" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="G150" s="2" t="inlineStr">
-        <is>
-          <t>AAJ-028</t>
-        </is>
-      </c>
-      <c r="H150" s="2" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
+          <t>3 - Medium</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr"/>
+      <c r="G150" s="2" t="inlineStr"/>
+      <c r="H150" s="2" t="inlineStr"/>
       <c r="I150" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -12090,23 +12054,257 @@
       <c r="M150" s="2" t="inlineStr"/>
       <c r="N150" s="4" t="inlineStr">
         <is>
+          <t>Ambang 1 + window panjang → simpan #1 (200) → simpan #2 kena 429 ×3 (1 asli + 2 retry, semua 429)</t>
+        </is>
+      </c>
+      <c r="O150" s="4" t="inlineStr">
+        <is>
+          <t>Toast "Terlalu banyak permintaan" tampil; jurnal #2 TIDAK tersimpan (daftar tetap 9 entri); sesi tetap aktif (429 ≠ logout)</t>
+        </is>
+      </c>
+      <c r="P150" s="4" t="inlineStr">
+        <is>
+          <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>TC-CFL-01</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Arus Kas</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>3 seksi arus kas</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>1 - Critical</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>AAJ-028</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M151" s="2" t="inlineStr"/>
+      <c r="N151" s="4" t="inlineStr">
+        <is>
+          <t>Buka laporan Arus Kas Maret</t>
+        </is>
+      </c>
+      <c r="O151" s="4" t="inlineStr">
+        <is>
+          <t>Seksi Operasi / Investasi / Pendanaan dengan subtotal; metode tidak langsung</t>
+        </is>
+      </c>
+      <c r="P151" s="4" t="inlineStr">
+        <is>
+          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>TC-CFL-02</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Arus Kas</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Konsistensi kas</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>1 - Critical</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>AAJ-028</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr"/>
+      <c r="N152" s="4" t="inlineStr">
+        <is>
+          <t>Cek formula</t>
+        </is>
+      </c>
+      <c r="O152" s="4" t="inlineStr">
+        <is>
+          <t>Kas akhir = kas awal + arus kas bersih (unit test)</t>
+        </is>
+      </c>
+      <c r="P152" s="4" t="inlineStr">
+        <is>
+          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>TC-CFL-03</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Arus Kas</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Mapping grup akun</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>2 - High</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>AAJ-028</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L153" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M153" s="2" t="inlineStr"/>
+      <c r="N153" s="4" t="inlineStr">
+        <is>
           <t>Ubah mapping di Pengaturan</t>
         </is>
       </c>
-      <c r="O150" s="4" t="inlineStr">
+      <c r="O153" s="4" t="inlineStr">
         <is>
           <t>Perubahan mapping tercermin di laporan</t>
         </is>
       </c>
-      <c r="P150" s="4" t="inlineStr">
+      <c r="P153" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P150"/>
-  <conditionalFormatting sqref="I2:I150">
+  <autoFilter ref="A1:P153"/>
+  <conditionalFormatting sqref="I2:I153">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
       <formula>$I2="Passed"</formula>
     </cfRule>
@@ -12159,7 +12357,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
@@ -12179,7 +12377,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5"/>

</xml_diff>

<commit_message>
feat(qa): --run-date override semua baris + regenerasi artefak 2026-08-19
- Generator: saat --run-date CLI, paksa Tanggal Run di SEMUA baris
  (bukan hanya baris kosong) — cegah check-qa-sync gagal karena
  perbedaan tanggal antara tracker on-disk dan hasil regenerasi
- Regenerasi artefak QA dengan QA_RUN_DATE=2026-08-19:
  tracker (152 baris), XLSX, testrail CSV, sample
- check-qa-sync PASS setelah commit ini

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/qa-test-cases-sample.xlsx
+++ b/qa-test-cases-sample.xlsx
@@ -682,7 +682,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -4738,7 +4738,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -5284,7 +5284,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
@@ -5674,7 +5674,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
@@ -6610,7 +6610,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
@@ -6688,7 +6688,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
@@ -6844,7 +6844,7 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
@@ -6922,7 +6922,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
@@ -7000,7 +7000,7 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -7390,7 +7390,7 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
@@ -7702,7 +7702,7 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -8162,7 +8162,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr">
@@ -8318,7 +8318,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr">
@@ -8396,7 +8396,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K102" s="2" t="inlineStr">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
@@ -8630,7 +8630,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr">
@@ -8786,7 +8786,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
@@ -8942,7 +8942,7 @@
       </c>
       <c r="J108" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K108" s="6" t="inlineStr">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="J111" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K111" s="6" t="inlineStr">
@@ -9254,7 +9254,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K113" s="2" t="inlineStr">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K115" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K116" s="2" t="inlineStr">
@@ -9644,7 +9644,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr">
@@ -9722,7 +9722,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr">
@@ -9800,7 +9800,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K120" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K121" s="2" t="inlineStr">
@@ -10034,7 +10034,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K122" s="2" t="inlineStr">
@@ -10112,7 +10112,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K124" s="2" t="inlineStr">
@@ -10268,7 +10268,7 @@
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K125" s="2" t="inlineStr">
@@ -10346,7 +10346,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K126" s="2" t="inlineStr">
@@ -10424,7 +10424,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K128" s="2" t="inlineStr">
@@ -10580,7 +10580,7 @@
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K129" s="2" t="inlineStr">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K130" s="2" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K131" s="2" t="inlineStr">
@@ -10814,7 +10814,7 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K132" s="2" t="inlineStr">
@@ -10892,7 +10892,7 @@
       </c>
       <c r="J133" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K133" s="2" t="inlineStr">
@@ -10970,7 +10970,7 @@
       </c>
       <c r="J134" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K134" s="6" t="inlineStr">
@@ -11048,7 +11048,7 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K135" s="2" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K136" s="2" t="inlineStr">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K138" s="2" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K139" s="2" t="inlineStr">
@@ -11378,7 +11378,7 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K140" s="2" t="inlineStr">
@@ -11444,7 +11444,7 @@
       </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K141" s="2" t="inlineStr">
@@ -11510,7 +11510,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
@@ -11642,7 +11642,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -11774,7 +11774,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr">
@@ -11840,7 +11840,7 @@
       </c>
       <c r="J147" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K147" s="2" t="inlineStr">
@@ -11906,7 +11906,7 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K148" s="2" t="inlineStr">
@@ -11972,7 +11972,7 @@
       </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K149" s="2" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K150" s="2" t="inlineStr">
@@ -12116,7 +12116,7 @@
       </c>
       <c r="J151" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K151" s="2" t="inlineStr">
@@ -12194,7 +12194,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">

</xml_diff>